<commit_message>
Add valueType column to DPEs
</commit_message>
<xml_diff>
--- a/linkage/data_processing_elements_linkage-NHANES11.xlsx
+++ b/linkage/data_processing_elements_linkage-NHANES11.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\twey\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41B2FE31-24FB-4E7A-900F-F2F63834FBD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A70CBD22-BA20-4543-BC6F-45B245E276CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{63444C23-9E00-4348-B1ED-05F831BC47B5}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Feuil1!$A$1:$M$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Feuil1!$A$1:$Q$23</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="119">
   <si>
     <t>index</t>
   </si>
@@ -396,6 +396,12 @@
   </si>
   <si>
     <t>Added in V2 of DataSchema.</t>
+  </si>
+  <si>
+    <t>valueType</t>
+  </si>
+  <si>
+    <t>text</t>
   </si>
 </sst>
 </file>
@@ -473,7 +479,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -500,6 +506,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -836,29 +845,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A96D0D0-036F-4639-8FBF-4A4CEF797E7C}">
-  <dimension ref="A1:P23"/>
+  <dimension ref="A1:Q23"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.42578125" style="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28.5703125" style="4" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="28.5703125" style="4" customWidth="1"/>
     <col min="4" max="4" width="59.28515625" style="5" customWidth="1"/>
-    <col min="5" max="5" width="14.5703125" style="4" customWidth="1"/>
-    <col min="6" max="6" width="14.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="43.5703125" style="4" customWidth="1"/>
-    <col min="8" max="8" width="44.85546875" style="5" customWidth="1"/>
-    <col min="9" max="9" width="24.42578125" style="3" customWidth="1"/>
-    <col min="10" max="10" width="12.85546875" style="3" customWidth="1"/>
-    <col min="11" max="11" width="18.85546875" style="3" customWidth="1"/>
-    <col min="12" max="12" width="16.7109375" style="3" customWidth="1"/>
-    <col min="13" max="13" width="57.42578125" style="3" customWidth="1"/>
-    <col min="14" max="14" width="22.28515625" style="3" customWidth="1"/>
-    <col min="15" max="15" width="29.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="30.28515625" style="3" customWidth="1"/>
-    <col min="17" max="16384" width="11.5703125" style="3"/>
+    <col min="5" max="5" width="11.5703125" style="10"/>
+    <col min="6" max="6" width="14.5703125" style="4" customWidth="1"/>
+    <col min="7" max="7" width="14.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="43.5703125" style="4" customWidth="1"/>
+    <col min="9" max="9" width="44.85546875" style="5" customWidth="1"/>
+    <col min="10" max="10" width="24.42578125" style="3" customWidth="1"/>
+    <col min="11" max="11" width="12.85546875" style="3" customWidth="1"/>
+    <col min="12" max="12" width="18.85546875" style="3" customWidth="1"/>
+    <col min="13" max="13" width="16.7109375" style="3" customWidth="1"/>
+    <col min="14" max="14" width="57.42578125" style="3" customWidth="1"/>
+    <col min="15" max="15" width="22.28515625" style="3" customWidth="1"/>
+    <col min="16" max="16" width="29.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="30.28515625" style="3" customWidth="1"/>
+    <col min="18" max="16384" width="11.5703125" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -872,43 +882,46 @@
         <v>17</v>
       </c>
       <c r="E1" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="F1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="I1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="J1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="K1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="L1" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="M1" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="N1" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="O1" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -921,26 +934,29 @@
       <c r="D2" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="E2" s="4" t="s">
-        <v>63</v>
+      <c r="E2" s="10" t="s">
+        <v>118</v>
       </c>
       <c r="F2" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G2" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="K2" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="L2" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="M2" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="N2" s="4" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -953,29 +969,32 @@
       <c r="D3" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="E3" s="4" t="s">
-        <v>63</v>
+      <c r="E3" s="10" t="s">
+        <v>118</v>
       </c>
       <c r="F3" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G3" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="K3" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="K3" s="4" t="s">
+      <c r="L3" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="L3" s="4" t="s">
+      <c r="M3" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="M3" s="4" t="s">
+      <c r="N3" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="P3" s="7" t="s">
+      <c r="Q3" s="7" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -988,29 +1007,32 @@
       <c r="D4" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="E4" s="4" t="s">
-        <v>63</v>
+      <c r="E4" s="10" t="s">
+        <v>118</v>
       </c>
       <c r="F4" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G4" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="K4" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="K4" s="4" t="s">
+      <c r="L4" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="L4" s="4" t="s">
+      <c r="M4" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="M4" s="4" t="s">
+      <c r="N4" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="P4" s="7" t="s">
+      <c r="Q4" s="7" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -1023,29 +1045,32 @@
       <c r="D5" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>63</v>
+      <c r="E5" s="10" t="s">
+        <v>118</v>
       </c>
       <c r="F5" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G5" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="J5" s="3" t="s">
+      <c r="K5" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="K5" s="4" t="s">
+      <c r="L5" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="L5" s="4" t="s">
+      <c r="M5" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="M5" s="4" t="s">
+      <c r="N5" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="P5" s="7" t="s">
+      <c r="Q5" s="7" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -1058,29 +1083,32 @@
       <c r="D6" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="E6" s="4" t="s">
-        <v>63</v>
+      <c r="E6" s="10" t="s">
+        <v>115</v>
       </c>
       <c r="F6" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G6" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="J6" s="3" t="s">
+      <c r="K6" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="K6" s="4" t="s">
+      <c r="L6" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="L6" s="4" t="s">
+      <c r="M6" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="M6" s="3">
+      <c r="N6" s="3">
         <v>2019</v>
       </c>
-      <c r="P6" s="7" t="s">
+      <c r="Q6" s="7" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -1093,29 +1121,32 @@
       <c r="D7" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="E7" s="4" t="s">
-        <v>63</v>
+      <c r="E7" s="10" t="s">
+        <v>115</v>
       </c>
       <c r="F7" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G7" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="J7" s="3" t="s">
+      <c r="K7" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="K7" s="4" t="s">
+      <c r="L7" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="L7" s="4" t="s">
+      <c r="M7" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="M7" s="4">
+      <c r="N7" s="4">
         <v>12</v>
       </c>
-      <c r="P7" s="7" t="s">
+      <c r="Q7" s="7" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -1128,35 +1159,38 @@
       <c r="D8" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="E8" s="4" t="s">
-        <v>63</v>
+      <c r="E8" s="10" t="s">
+        <v>115</v>
       </c>
       <c r="F8" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G8" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="H8" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="H8" s="5" t="s">
+      <c r="I8" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="J8" s="3" t="s">
+      <c r="K8" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="K8" s="4" t="s">
+      <c r="L8" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="L8" s="4" t="s">
-        <v>89</v>
       </c>
       <c r="M8" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="P8" s="7" t="s">
+      <c r="N8" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="Q8" s="7" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -1169,35 +1203,38 @@
       <c r="D9" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="E9" s="4" t="s">
-        <v>63</v>
+      <c r="E9" s="10" t="s">
+        <v>115</v>
       </c>
       <c r="F9" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G9" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="I9" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="J9" s="3" t="s">
+      <c r="K9" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="K9" s="3" t="s">
+      <c r="L9" s="3" t="s">
         <v>45</v>
-      </c>
-      <c r="L9" s="3" t="s">
-        <v>44</v>
       </c>
       <c r="M9" s="3" t="s">
         <v>44</v>
       </c>
       <c r="N9" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="O9" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="P9" s="7" t="s">
+      <c r="Q9" s="7" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>9</v>
       </c>
@@ -1210,35 +1247,38 @@
       <c r="D10" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="E10" s="4" t="s">
-        <v>63</v>
+      <c r="E10" s="10" t="s">
+        <v>115</v>
       </c>
       <c r="F10" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G10" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="H10" s="5" t="s">
+      <c r="I10" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="J10" s="3" t="s">
+      <c r="K10" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="K10" s="3" t="s">
+      <c r="L10" s="3" t="s">
         <v>45</v>
-      </c>
-      <c r="L10" s="4" t="s">
-        <v>44</v>
       </c>
       <c r="M10" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="N10" s="3" t="s">
+      <c r="N10" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="O10" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="P10" s="7" t="s">
+      <c r="Q10" s="7" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -1251,29 +1291,32 @@
       <c r="D11" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="E11" s="4" t="s">
-        <v>63</v>
+      <c r="E11" s="10" t="s">
+        <v>115</v>
       </c>
       <c r="F11" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G11" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="H11" s="5" t="s">
+      <c r="I11" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="J11" s="3" t="s">
+      <c r="K11" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="K11" s="4" t="s">
+      <c r="L11" s="4" t="s">
         <v>45</v>
-      </c>
-      <c r="L11" s="4" t="s">
-        <v>44</v>
       </c>
       <c r="M11" s="4" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="12" spans="1:16" ht="90" x14ac:dyDescent="0.25">
+      <c r="N11" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" ht="90" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>11</v>
       </c>
@@ -1286,35 +1329,38 @@
       <c r="D12" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="E12" s="4" t="s">
-        <v>63</v>
+      <c r="E12" s="10" t="s">
+        <v>115</v>
       </c>
       <c r="F12" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G12" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="G12" s="5" t="s">
+      <c r="H12" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="H12" s="5" t="s">
+      <c r="I12" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="J12" s="9" t="s">
+      <c r="K12" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="K12" s="4" t="s">
+      <c r="L12" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="L12" s="4" t="s">
-        <v>89</v>
       </c>
       <c r="M12" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="P12" s="9" t="s">
+      <c r="N12" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="Q12" s="9" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -1327,29 +1373,29 @@
       <c r="D13" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="E13" s="4" t="s">
-        <v>63</v>
+      <c r="E13" s="10" t="s">
+        <v>118</v>
       </c>
       <c r="F13" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G13" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="H13" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="J13" s="3" t="s">
+      <c r="K13" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="K13" s="4" t="s">
+      <c r="L13" s="4" t="s">
         <v>45</v>
-      </c>
-      <c r="L13" s="4" t="s">
-        <v>44</v>
       </c>
       <c r="M13" s="4" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="14" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+      <c r="N13" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -1362,32 +1408,35 @@
       <c r="D14" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="E14" s="4" t="s">
-        <v>63</v>
+      <c r="E14" s="10" t="s">
+        <v>115</v>
       </c>
       <c r="F14" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G14" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="G14" s="5" t="s">
+      <c r="H14" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="H14" s="5" t="s">
+      <c r="I14" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="J14" s="3" t="s">
+      <c r="K14" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="K14" s="4" t="s">
+      <c r="L14" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="L14" s="4" t="s">
+      <c r="M14" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="M14" s="5" t="s">
+      <c r="N14" s="5" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:17" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -1400,35 +1449,38 @@
       <c r="D15" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="E15" s="4" t="s">
-        <v>63</v>
+      <c r="E15" s="10" t="s">
+        <v>115</v>
       </c>
       <c r="F15" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G15" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="G15" s="5" t="s">
+      <c r="H15" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="H15" s="5" t="s">
+      <c r="I15" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="J15" s="3" t="s">
+      <c r="K15" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="K15" s="4" t="s">
+      <c r="L15" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="L15" s="4" t="s">
+      <c r="M15" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="M15" s="5" t="s">
+      <c r="N15" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="P15" s="7" t="s">
+      <c r="Q15" s="7" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:17" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>15</v>
       </c>
@@ -1441,32 +1493,35 @@
       <c r="D16" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="E16" s="4" t="s">
-        <v>63</v>
+      <c r="E16" s="10" t="s">
+        <v>115</v>
       </c>
       <c r="F16" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G16" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="G16" s="5" t="s">
+      <c r="H16" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="H16" s="5" t="s">
+      <c r="I16" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="J16" s="3" t="s">
+      <c r="K16" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="K16" s="4" t="s">
+      <c r="L16" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="L16" s="4" t="s">
+      <c r="M16" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="M16" s="5" t="s">
+      <c r="N16" s="5" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="17" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:17" ht="45" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>16</v>
       </c>
@@ -1479,32 +1534,35 @@
       <c r="D17" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="E17" s="4" t="s">
-        <v>63</v>
+      <c r="E17" s="10" t="s">
+        <v>115</v>
       </c>
       <c r="F17" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G17" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="G17" s="5" t="s">
+      <c r="H17" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="H17" s="5" t="s">
+      <c r="I17" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="J17" s="3" t="s">
+      <c r="K17" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="K17" s="4" t="s">
+      <c r="L17" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="L17" s="4" t="s">
+      <c r="M17" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="M17" s="5" t="s">
+      <c r="N17" s="5" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:17" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>17</v>
       </c>
@@ -1517,32 +1575,35 @@
       <c r="D18" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="E18" s="4" t="s">
-        <v>63</v>
+      <c r="E18" s="10" t="s">
+        <v>115</v>
       </c>
       <c r="F18" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G18" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="G18" s="5" t="s">
+      <c r="H18" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="H18" s="5" t="s">
+      <c r="I18" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="J18" s="3" t="s">
+      <c r="K18" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="K18" s="4" t="s">
+      <c r="L18" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="L18" s="4" t="s">
+      <c r="M18" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="M18" s="5" t="s">
+      <c r="N18" s="5" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="19" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:17" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -1555,32 +1616,35 @@
       <c r="D19" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="E19" s="4" t="s">
-        <v>63</v>
+      <c r="E19" s="10" t="s">
+        <v>115</v>
       </c>
       <c r="F19" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G19" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="G19" s="5" t="s">
+      <c r="H19" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="H19" s="5" t="s">
+      <c r="I19" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="J19" s="3" t="s">
+      <c r="K19" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="K19" s="4" t="s">
+      <c r="L19" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="L19" s="4" t="s">
+      <c r="M19" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="M19" s="5" t="s">
+      <c r="N19" s="5" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="20" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:17" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>19</v>
       </c>
@@ -1593,32 +1657,35 @@
       <c r="D20" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="E20" s="4" t="s">
-        <v>63</v>
+      <c r="E20" s="10" t="s">
+        <v>115</v>
       </c>
       <c r="F20" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G20" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="G20" s="5" t="s">
+      <c r="H20" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="H20" s="5" t="s">
+      <c r="I20" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="J20" s="3" t="s">
+      <c r="K20" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="K20" s="4" t="s">
+      <c r="L20" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="L20" s="4" t="s">
+      <c r="M20" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="M20" s="5" t="s">
+      <c r="N20" s="5" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="21" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:17" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>20</v>
       </c>
@@ -1631,32 +1698,35 @@
       <c r="D21" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="E21" s="4" t="s">
-        <v>63</v>
+      <c r="E21" s="10" t="s">
+        <v>115</v>
       </c>
       <c r="F21" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G21" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="G21" s="5" t="s">
+      <c r="H21" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="H21" s="5" t="s">
+      <c r="I21" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="J21" s="3" t="s">
+      <c r="K21" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="K21" s="4" t="s">
+      <c r="L21" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="L21" s="4" t="s">
+      <c r="M21" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="M21" s="5" t="s">
+      <c r="N21" s="5" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="22" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:17" ht="45" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
         <v>21</v>
       </c>
@@ -1669,32 +1739,35 @@
       <c r="D22" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="E22" s="4" t="s">
-        <v>63</v>
+      <c r="E22" s="10" t="s">
+        <v>115</v>
       </c>
       <c r="F22" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G22" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="G22" s="5" t="s">
+      <c r="H22" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="H22" s="5" t="s">
+      <c r="I22" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="J22" s="3" t="s">
+      <c r="K22" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="K22" s="4" t="s">
+      <c r="L22" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="L22" s="4" t="s">
+      <c r="M22" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="M22" s="5" t="s">
+      <c r="N22" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="23" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:17" ht="45" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>22</v>
       </c>
@@ -1707,32 +1780,39 @@
       <c r="D23" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="E23" s="4" t="s">
-        <v>63</v>
+      <c r="E23" s="10" t="s">
+        <v>115</v>
       </c>
       <c r="F23" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G23" s="4" t="s">
         <v>60</v>
       </c>
       <c r="H23" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I23" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="J23" s="3" t="s">
+      <c r="K23" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="K23" s="4" t="s">
+      <c r="L23" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="L23" s="4" t="s">
+      <c r="M23" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="M23" s="5" t="s">
+      <c r="N23" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="P23" s="7" t="s">
+      <c r="Q23" s="7" t="s">
         <v>94</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:Q23" xr:uid="{2A96D0D0-036F-4639-8FBF-4A4CEF797E7C}"/>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>